<commit_message>
añado resultados de pruebas
</commit_message>
<xml_diff>
--- a/Pruebas cohorte general I/con KNN n=3/resultados_pruebas_CON_KNN_n3.xlsx
+++ b/Pruebas cohorte general I/con KNN n=3/resultados_pruebas_CON_KNN_n3.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\TFG\Pruebas cohorte general I\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\TFG\Pruebas cohorte general I\con KNN n=3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26158792-EA06-444F-9873-5A33BBD3F8BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8589B814-F442-4F1E-9848-CE93585A6317}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="750" yWindow="525" windowWidth="27510" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
   <si>
     <t>Modelo</t>
   </si>
@@ -49,6 +49,24 @@
   </si>
   <si>
     <t>LightGBM</t>
+  </si>
+  <si>
+    <t>error</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.7702</t>
+  </si>
+  <si>
+    <t>nan</t>
+  </si>
+  <si>
+    <t>0.7732 ± 0.009</t>
+  </si>
+  <si>
+    <t>0.7838 ± 0.0088</t>
+  </si>
+  <si>
+    <t>0.7848</t>
   </si>
 </sst>
 </file>
@@ -58,7 +76,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -73,11 +91,6 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
@@ -141,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -152,17 +165,20 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -468,42 +484,62 @@
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="3"/>
+      <c r="B2" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="3"/>
+      <c r="B3" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3">
+        <v>0.77249999999999996</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="3"/>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="5"/>
+      <c r="B5" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="3"/>
+      <c r="B6" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="7"/>
+      <c r="B8" s="5"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="6"/>
+      <c r="B11" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>